<commit_message>
Conversión de la distancia a tipo Double y almacenamiento estructurado de los resultados en Excel para facilitar el análisis y explotación posterior de los datos.
</commit_message>
<xml_diff>
--- a/Resultado_Negocios.xlsx
+++ b/Resultado_Negocios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\desarrollo\UiPath\ObtenerDistanciaTiempo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED2FC080-05C6-4158-8C84-956B85E515D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7BFA74-08F2-4F26-947A-CAB56F550A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9795" yWindow="-14670" windowWidth="18330" windowHeight="11745" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Peluqueria Alcobendas (4)" sheetId="7" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="Hipica madrid norte" sheetId="11" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">HipicasMadridNorte!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">HipicasMadridNorte!$A$1:$L$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Peluqueria Alcobendas (4)'!$A$1:$C$96</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1450" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="496">
   <si>
     <t>Nombre</t>
   </si>
@@ -1448,22 +1448,79 @@
     <t>Carr. de Soto del Real a, M608, Km 13, 500, 28791 Guadalix de la Sierra, Madrid</t>
   </si>
   <si>
+    <t>Origen</t>
+  </si>
+  <si>
+    <t>Distancia</t>
+  </si>
+  <si>
+    <t>Tiempo</t>
+  </si>
+  <si>
+    <t>Lavanderia Bloomest Alcobendas Norte, C. de Ruperto Chapí, 57, LOCAL, 28100 Alcobendas, Madrid</t>
+  </si>
+  <si>
+    <t>28 min</t>
+  </si>
+  <si>
+    <t>31 min</t>
+  </si>
+  <si>
+    <t>30 min</t>
+  </si>
+  <si>
+    <t>38 min</t>
+  </si>
+  <si>
+    <t>40 min</t>
+  </si>
+  <si>
+    <t>44 min</t>
+  </si>
+  <si>
+    <t>36 min</t>
+  </si>
+  <si>
+    <t>45 min</t>
+  </si>
+  <si>
+    <t>1 h 7 min</t>
+  </si>
+  <si>
+    <t>13 min</t>
+  </si>
+  <si>
+    <t>1 h 4 min</t>
+  </si>
+  <si>
+    <t>39 min</t>
+  </si>
+  <si>
+    <t>29 min</t>
+  </si>
+  <si>
+    <t>1 h 3 min</t>
+  </si>
+  <si>
+    <t>1 h 29 min</t>
+  </si>
+  <si>
+    <t>34 min</t>
+  </si>
+  <si>
+    <t>1 h 24 min</t>
+  </si>
+  <si>
+    <t>22 min</t>
+  </si>
+  <si>
+    <t>33 min</t>
+  </si>
+  <si>
     <t>Hipicas.net</t>
   </si>
   <si>
     <t>Av. de Alberto Alcocer, 49, Chamartín, 28016 Madrid</t>
-  </si>
-  <si>
-    <t>Lavanderia Bloomest Alcobendas Norte, C. de Ruperto Chapí, 57, LOCAL, 28100 Alcobendas, Madrid</t>
-  </si>
-  <si>
-    <t>Origen</t>
-  </si>
-  <si>
-    <t>Tiempo</t>
-  </si>
-  <si>
-    <t>Distancia</t>
   </si>
 </sst>
 </file>
@@ -6732,12 +6789,13 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.109375" customWidth="1"/>
+    <col min="3" max="3" width="74" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="11" width="8.88671875" customWidth="1"/>
@@ -6755,13 +6813,13 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="E1" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="F1" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -6775,7 +6833,13 @@
         <v>413</v>
       </c>
       <c r="D2" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E2">
+        <v>22.1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -6789,7 +6853,13 @@
         <v>361</v>
       </c>
       <c r="D3" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E3">
+        <v>30.4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -6803,7 +6873,13 @@
         <v>355</v>
       </c>
       <c r="D4" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E4">
+        <v>22.3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -6817,7 +6893,13 @@
         <v>384</v>
       </c>
       <c r="D5" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E5">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="F5" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -6831,7 +6913,13 @@
         <v>370</v>
       </c>
       <c r="D6" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E6">
+        <v>33.9</v>
+      </c>
+      <c r="F6" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -6845,7 +6933,13 @@
         <v>346</v>
       </c>
       <c r="D7" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E7">
+        <v>34.4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -6859,7 +6953,13 @@
         <v>343</v>
       </c>
       <c r="D8" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E8">
+        <v>41.9</v>
+      </c>
+      <c r="F8" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -6873,7 +6973,13 @@
         <v>364</v>
       </c>
       <c r="D9" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E9">
+        <v>27.3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -6887,7 +6993,13 @@
         <v>381</v>
       </c>
       <c r="D10" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E10">
+        <v>27.3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>481</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -6901,10 +7013,16 @@
         <v>431</v>
       </c>
       <c r="D11" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E11">
+        <v>42.7</v>
+      </c>
+      <c r="F11" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>468</v>
       </c>
@@ -6915,7 +7033,13 @@
         <v>470</v>
       </c>
       <c r="D12" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E12">
+        <v>74.400000000000006</v>
+      </c>
+      <c r="F12" t="s">
+        <v>483</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -6929,10 +7053,16 @@
         <v>396</v>
       </c>
       <c r="D13" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
+      </c>
+      <c r="F13" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>426</v>
       </c>
@@ -6943,7 +7073,13 @@
         <v>428</v>
       </c>
       <c r="D14" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E14">
+        <v>80</v>
+      </c>
+      <c r="F14" t="s">
+        <v>485</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -6957,7 +7093,13 @@
         <v>375</v>
       </c>
       <c r="D15" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E15">
+        <v>39.6</v>
+      </c>
+      <c r="F15" t="s">
+        <v>486</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -6971,10 +7113,16 @@
         <v>404</v>
       </c>
       <c r="D16" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E16">
+        <v>24.8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>441</v>
       </c>
@@ -6985,10 +7133,16 @@
         <v>443</v>
       </c>
       <c r="D17" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E17">
+        <v>79.599999999999994</v>
+      </c>
+      <c r="F17" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>405</v>
       </c>
@@ -6999,10 +7153,16 @@
         <v>407</v>
       </c>
       <c r="D18" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E18">
+        <v>101</v>
+      </c>
+      <c r="F18" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>353</v>
       </c>
@@ -7013,10 +7173,16 @@
         <v>355</v>
       </c>
       <c r="D19" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E19">
+        <v>22.3</v>
+      </c>
+      <c r="F19" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>388</v>
       </c>
@@ -7027,10 +7193,16 @@
         <v>390</v>
       </c>
       <c r="D20" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E20">
+        <v>27.3</v>
+      </c>
+      <c r="F20" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>391</v>
       </c>
@@ -7041,10 +7213,16 @@
         <v>393</v>
       </c>
       <c r="D21" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E21">
+        <v>26.1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>397</v>
       </c>
@@ -7055,10 +7233,16 @@
         <v>398</v>
       </c>
       <c r="D22" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E22">
+        <v>32.4</v>
+      </c>
+      <c r="F22" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>338</v>
       </c>
@@ -7069,10 +7253,16 @@
         <v>340</v>
       </c>
       <c r="D23" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E23">
+        <v>33.6</v>
+      </c>
+      <c r="F23" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>365</v>
       </c>
@@ -7083,10 +7273,16 @@
         <v>367</v>
       </c>
       <c r="D24" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E24">
+        <v>30.4</v>
+      </c>
+      <c r="F24" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>417</v>
       </c>
@@ -7097,10 +7293,16 @@
         <v>419</v>
       </c>
       <c r="D25" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E25">
+        <v>85.6</v>
+      </c>
+      <c r="F25" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>335</v>
       </c>
@@ -7111,10 +7313,16 @@
         <v>337</v>
       </c>
       <c r="D26" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E26">
+        <v>32.9</v>
+      </c>
+      <c r="F26" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>423</v>
       </c>
@@ -7125,10 +7333,16 @@
         <v>425</v>
       </c>
       <c r="D27" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E27">
+        <v>33.6</v>
+      </c>
+      <c r="F27" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>350</v>
       </c>
@@ -7139,10 +7353,16 @@
         <v>352</v>
       </c>
       <c r="D28" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E28">
+        <v>10.4</v>
+      </c>
+      <c r="F28" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>385</v>
       </c>
@@ -7153,10 +7373,16 @@
         <v>387</v>
       </c>
       <c r="D29" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E29">
+        <v>26.3</v>
+      </c>
+      <c r="F29" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>347</v>
       </c>
@@ -7167,10 +7393,16 @@
         <v>349</v>
       </c>
       <c r="D30" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E30">
+        <v>21.9</v>
+      </c>
+      <c r="F30" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>465</v>
       </c>
@@ -7181,24 +7413,36 @@
         <v>466</v>
       </c>
       <c r="D31" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E31">
+        <v>18.7</v>
+      </c>
+      <c r="F31" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>471</v>
+        <v>494</v>
       </c>
       <c r="B32" t="s">
         <v>165</v>
       </c>
       <c r="C32" t="s">
-        <v>472</v>
+        <v>495</v>
       </c>
       <c r="D32" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E32">
+        <v>27.6</v>
+      </c>
+      <c r="F32" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>356</v>
       </c>
@@ -7209,10 +7453,16 @@
         <v>358</v>
       </c>
       <c r="D33" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E33">
+        <v>22.1</v>
+      </c>
+      <c r="F33" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>376</v>
       </c>
@@ -7223,10 +7473,16 @@
         <v>378</v>
       </c>
       <c r="D34" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+        <v>474</v>
+      </c>
+      <c r="E34">
+        <v>22.2</v>
+      </c>
+      <c r="F34" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>414</v>
       </c>
@@ -7237,14 +7493,35 @@
         <v>416</v>
       </c>
       <c r="D35" t="s">
-        <v>473</v>
+        <v>474</v>
+      </c>
+      <c r="E35">
+        <v>11.2</v>
+      </c>
+      <c r="F35" t="s">
+        <v>492</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1" xr:uid="{00000000-0001-0000-0700-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L101">
-      <sortCondition ref="A1"/>
-    </sortState>
+  <autoFilter ref="A1:L35" xr:uid="{00000000-0009-0000-0000-000008000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="13 min"/>
+        <filter val="22 min"/>
+        <filter val="28 min"/>
+        <filter val="29 min"/>
+        <filter val="30 min"/>
+        <filter val="31 min"/>
+        <filter val="33 min"/>
+        <filter val="34 min"/>
+        <filter val="36 min"/>
+        <filter val="38 min"/>
+        <filter val="39 min"/>
+        <filter val="40 min"/>
+        <filter val="44 min"/>
+        <filter val="45 min"/>
+      </filters>
+    </filterColumn>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>

</xml_diff>